<commit_message>
added tests and 404 page
</commit_message>
<xml_diff>
--- a/authtest/src/test/resources/digital/places/root/test.xlsx
+++ b/authtest/src/test/resources/digital/places/root/test.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9975" windowHeight="1605"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9975" windowHeight="1605" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="nlivalid" sheetId="1" r:id="rId1"/>
@@ -43,10 +43,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -69,13 +77,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -354,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -368,14 +379,18 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -383,6 +398,9 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>